<commit_message>
docs: update example data in README and demo sheet
</commit_message>
<xml_diff>
--- a/demo-sheet.xlsx
+++ b/demo-sheet.xlsx
@@ -398,11 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C16"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="62.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -423,7 +418,7 @@
         <v>Rahim Uddin</v>
       </c>
       <c r="C2" t="str">
-        <v>https://github.com/ALPHAMAN-0/zenji_shop</v>
+        <v>https://github.com/octocat/Hello-World</v>
       </c>
     </row>
     <row r="3">
@@ -434,7 +429,7 @@
         <v>Nusrat Jahan</v>
       </c>
       <c r="C3" t="str">
-        <v>https://github.com/ALPHAMAN-0/parcelFlow_Frontend</v>
+        <v>https://github.com/octocat/Spoon-Knife</v>
       </c>
     </row>
     <row r="4">
@@ -445,7 +440,7 @@
         <v>Tanvir Ahmed</v>
       </c>
       <c r="C4" t="str">
-        <v>https://github.com/ALPHAMAN-0/Gridwise_LLM_Energy_Optimizer</v>
+        <v>github.com/octocat/octocat.github.io</v>
       </c>
     </row>
     <row r="5">
@@ -456,7 +451,7 @@
         <v>Farhana Akter</v>
       </c>
       <c r="C5" t="str">
-        <v>github.com/ALPHAMAN-0/crawler-atlas</v>
+        <v>https://github.com/octocat/Hello-World</v>
       </c>
     </row>
     <row r="6">
@@ -467,7 +462,7 @@
         <v>Sabbir Hossain</v>
       </c>
       <c r="C6" t="str">
-        <v>https://github.com/ALPHAMAN-0/DailyMedicineTracker</v>
+        <v>https://github.com/octocat/Spoon-Knife</v>
       </c>
     </row>
     <row r="7">
@@ -478,7 +473,7 @@
         <v>Sumaiya Islam</v>
       </c>
       <c r="C7" t="str">
-        <v>https://github.com/ALPHAMAN-0/Unlimited_Storage</v>
+        <v>github.com/octocat/octocat.github.io</v>
       </c>
     </row>
     <row r="8">
@@ -489,7 +484,7 @@
         <v>Arif Rahman</v>
       </c>
       <c r="C8" t="str">
-        <v>https://github.com/ALPHAMAN-0/MEAN</v>
+        <v>https://github.com/octocat/Hello-World</v>
       </c>
     </row>
     <row r="9">
@@ -500,7 +495,7 @@
         <v>Tasnim Sultana</v>
       </c>
       <c r="C9" t="str">
-        <v>https://github.com/ALPHAMAN-0/AboutMe</v>
+        <v>https://github.com/octocat/Spoon-Knife</v>
       </c>
     </row>
     <row r="10">
@@ -511,7 +506,7 @@
         <v>Rakib Chowdhury</v>
       </c>
       <c r="C10" t="str">
-        <v>https://github.com/ALPHAMAN-0/AIUB_NOTICE_BOARD</v>
+        <v>github.com/octocat/octocat.github.io</v>
       </c>
     </row>
     <row r="11">
@@ -522,7 +517,7 @@
         <v>Jannatul Ferdous</v>
       </c>
       <c r="C11" t="str">
-        <v>https://github.com/ALPHAMAN-0/CV_Management</v>
+        <v>https://github.com/octocat/Hello-World</v>
       </c>
     </row>
     <row r="12">
@@ -533,7 +528,7 @@
         <v>Shakil Mahmud</v>
       </c>
       <c r="C12" t="str">
-        <v>github.com/ALPHAMAN-0/Order_Tracking_Screen</v>
+        <v>github.com/octocat/Spoon-Knife</v>
       </c>
     </row>
     <row r="13">
@@ -544,7 +539,7 @@
         <v>Lamia Tabassum</v>
       </c>
       <c r="C13" t="str">
-        <v>https://github.com/ALPHAMAN-0/Sir_ar_last_date</v>
+        <v>https://github.com/octocat/octocat.github.io</v>
       </c>
     </row>
     <row r="14">
@@ -555,7 +550,7 @@
         <v>Nayeem Sarker</v>
       </c>
       <c r="C14" t="str">
-        <v>https://github.com/ALPHAMAN-0/My_Programming_Lab</v>
+        <v>https://github.com/octocat/Hello-World</v>
       </c>
     </row>
     <row r="15">
@@ -566,7 +561,7 @@
         <v>Fahim Morshed</v>
       </c>
       <c r="C15" t="str">
-        <v>https://github.com/ALPHAMAN-0/task-1-not-here</v>
+        <v>https://github.com/octocat/this-repo-does-not-exist-12345</v>
       </c>
     </row>
     <row r="16">

</xml_diff>